<commit_message>
Actualizacion datos REM 2026-07-06 09:39 (orquestador)
</commit_message>
<xml_diff>
--- a/output/2024_A24_SECCION_E_TABLAS.xlsx
+++ b/output/2024_A24_SECCION_E_TABLAS.xlsx
@@ -184,16 +184,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -209,7 +201,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -217,31 +209,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -543,48 +517,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -625,7 +599,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3">
@@ -666,7 +640,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4">
@@ -707,7 +681,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5">
@@ -748,7 +722,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6">
@@ -789,7 +763,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
       <c r="B7">
@@ -830,7 +804,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8">
@@ -884,48 +858,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -966,7 +940,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3">
@@ -1007,7 +981,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4">
@@ -1048,7 +1022,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5">
@@ -1089,7 +1063,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6">
@@ -1130,7 +1104,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
       <c r="B7">
@@ -1171,7 +1145,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8">
@@ -1225,48 +1199,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -1307,7 +1281,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>21</v>
       </c>
       <c r="B3">
@@ -1348,7 +1322,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4">
@@ -1389,7 +1363,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
       <c r="B5">
@@ -1430,7 +1404,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>24</v>
       </c>
       <c r="B6">
@@ -1471,7 +1445,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>25</v>
       </c>
       <c r="B7">
@@ -1512,7 +1486,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>26</v>
       </c>
       <c r="B8">
@@ -1553,7 +1527,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>27</v>
       </c>
       <c r="B9">
@@ -1594,7 +1568,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>28</v>
       </c>
       <c r="B10">
@@ -1635,7 +1609,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>29</v>
       </c>
       <c r="B11">
@@ -1676,7 +1650,7 @@
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>30</v>
       </c>
       <c r="B12">
@@ -1717,7 +1691,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>31</v>
       </c>
       <c r="B13">
@@ -1758,7 +1732,7 @@
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
+      <c r="A14" t="s">
         <v>32</v>
       </c>
       <c r="B14">
@@ -1799,7 +1773,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
       <c r="B15">
@@ -1840,7 +1814,7 @@
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="2" t="s">
+      <c r="A16" t="s">
         <v>34</v>
       </c>
       <c r="B16">
@@ -1894,48 +1868,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -1976,7 +1950,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>21</v>
       </c>
       <c r="B3">
@@ -2017,7 +1991,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4">
@@ -2052,7 +2026,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
       <c r="B5">
@@ -2093,7 +2067,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>24</v>
       </c>
       <c r="B6">
@@ -2134,7 +2108,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>25</v>
       </c>
       <c r="B7">
@@ -2175,7 +2149,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>26</v>
       </c>
       <c r="B8">
@@ -2216,7 +2190,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>27</v>
       </c>
       <c r="B9">
@@ -2251,7 +2225,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>28</v>
       </c>
       <c r="B10">
@@ -2292,7 +2266,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>29</v>
       </c>
       <c r="B11">
@@ -2333,7 +2307,7 @@
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>30</v>
       </c>
       <c r="B12">
@@ -2374,7 +2348,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>31</v>
       </c>
       <c r="B13">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
+      <c r="A14" t="s">
         <v>32</v>
       </c>
       <c r="B14">
@@ -2456,7 +2430,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
       <c r="B15">
@@ -2497,7 +2471,7 @@
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="2" t="s">
+      <c r="A16" t="s">
         <v>34</v>
       </c>
       <c r="B16">
@@ -2551,48 +2525,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -2633,7 +2607,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>36</v>
       </c>
       <c r="B3">
@@ -2674,7 +2648,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>37</v>
       </c>
       <c r="B4">
@@ -2715,7 +2689,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>38</v>
       </c>
       <c r="B5">
@@ -2756,7 +2730,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
       <c r="B6">
@@ -2797,7 +2771,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7">
@@ -2838,7 +2812,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
       <c r="B8">
@@ -2879,7 +2853,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>42</v>
       </c>
       <c r="B9">
@@ -2920,7 +2894,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>43</v>
       </c>
       <c r="B10">
@@ -2961,7 +2935,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>44</v>
       </c>
       <c r="B11">
@@ -3002,7 +2976,7 @@
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>45</v>
       </c>
       <c r="B12">
@@ -3043,7 +3017,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>46</v>
       </c>
       <c r="B13">
@@ -3084,7 +3058,7 @@
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
+      <c r="A14" t="s">
         <v>47</v>
       </c>
       <c r="B14">
@@ -3125,7 +3099,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>48</v>
       </c>
       <c r="B15">
@@ -3166,7 +3140,7 @@
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="2" t="s">
+      <c r="A16" t="s">
         <v>49</v>
       </c>
       <c r="B16">
@@ -3207,7 +3181,7 @@
       </c>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="2" t="s">
+      <c r="A17" t="s">
         <v>50</v>
       </c>
       <c r="B17">
@@ -3248,7 +3222,7 @@
       </c>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="2" t="s">
+      <c r="A18" t="s">
         <v>51</v>
       </c>
       <c r="B18">
@@ -3302,48 +3276,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
@@ -3384,7 +3358,7 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>36</v>
       </c>
       <c r="B3">
@@ -3425,7 +3399,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>37</v>
       </c>
       <c r="B4">
@@ -3466,7 +3440,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>38</v>
       </c>
       <c r="B5">
@@ -3501,7 +3475,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
       <c r="B6">
@@ -3542,7 +3516,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7">
@@ -3583,7 +3557,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
       <c r="B8">
@@ -3624,7 +3598,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>42</v>
       </c>
       <c r="B9">
@@ -3665,7 +3639,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>43</v>
       </c>
       <c r="B10">
@@ -3706,7 +3680,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>44</v>
       </c>
       <c r="B11">
@@ -3747,7 +3721,7 @@
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>45</v>
       </c>
       <c r="B12">
@@ -3788,7 +3762,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>46</v>
       </c>
       <c r="B13">
@@ -3829,7 +3803,7 @@
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
+      <c r="A14" t="s">
         <v>47</v>
       </c>
       <c r="B14">
@@ -3870,7 +3844,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>48</v>
       </c>
       <c r="B15">
@@ -3911,7 +3885,7 @@
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="2" t="s">
+      <c r="A16" t="s">
         <v>49</v>
       </c>
       <c r="B16">
@@ -3952,7 +3926,7 @@
       </c>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="2" t="s">
+      <c r="A17" t="s">
         <v>50</v>
       </c>
       <c r="B17">
@@ -3993,7 +3967,7 @@
       </c>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="2" t="s">
+      <c r="A18" t="s">
         <v>51</v>
       </c>
       <c r="B18">

</xml_diff>